<commit_message>
mejoras del logico etc
</commit_message>
<xml_diff>
--- a/normalizacion/NORMALIZACION_BD_NIKE_GRUPO_5.xlsx
+++ b/normalizacion/NORMALIZACION_BD_NIKE_GRUPO_5.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1IDT\CI2\diseño_base_datos\proyecto_parcial\workspace-01a17fea-688d-7d0a-8783-64568db11e38\proyecto_parcial\normalizacion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1IDT\CI2\diseño_base_datos\proyecto_parcial\normalizacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EEFA74D-8D35-4C3B-B5AB-B3B026E663F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8C69B0F-DB3B-412C-B466-8CED7BA4E41C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0FN" sheetId="1" r:id="rId1"/>
@@ -799,18 +799,8 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -822,21 +812,35 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -844,14 +848,10 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1184,56 +1184,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-      <c r="L1" s="6"/>
-      <c r="M1" s="6"/>
-      <c r="N1" s="6"/>
-      <c r="O1" s="6"/>
-      <c r="P1" s="6"/>
-      <c r="Q1" s="6"/>
-      <c r="R1" s="6"/>
-      <c r="S1" s="6"/>
-      <c r="T1" s="6"/>
-      <c r="U1" s="6"/>
-      <c r="V1" s="6"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="P1" s="17"/>
+      <c r="Q1" s="17"/>
+      <c r="R1" s="17"/>
+      <c r="S1" s="17"/>
+      <c r="T1" s="17"/>
+      <c r="U1" s="17"/>
+      <c r="V1" s="17"/>
     </row>
     <row r="3" spans="1:22" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="10"/>
-      <c r="Q3" s="10"/>
-      <c r="R3" s="10"/>
-      <c r="S3" s="10"/>
-      <c r="T3" s="10"/>
-      <c r="U3" s="10"/>
-      <c r="V3" s="10"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
+      <c r="M3" s="18"/>
+      <c r="N3" s="18"/>
+      <c r="O3" s="18"/>
+      <c r="P3" s="18"/>
+      <c r="Q3" s="18"/>
+      <c r="R3" s="18"/>
+      <c r="S3" s="18"/>
+      <c r="T3" s="18"/>
+      <c r="U3" s="18"/>
+      <c r="V3" s="18"/>
     </row>
     <row r="4" spans="1:22" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -1272,7 +1272,7 @@
       <c r="L4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="M4" s="9" t="s">
+      <c r="M4" s="6" t="s">
         <v>14</v>
       </c>
       <c r="N4" s="1" t="s">
@@ -1307,7 +1307,7 @@
       <c r="A5" s="2">
         <v>9001</v>
       </c>
-      <c r="B5" s="26">
+      <c r="B5" s="16">
         <v>46300</v>
       </c>
       <c r="C5" s="3">
@@ -1364,10 +1364,10 @@
       <c r="T5" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="U5" s="26">
+      <c r="U5" s="16">
         <v>46301</v>
       </c>
-      <c r="V5" s="25" t="s">
+      <c r="V5" s="15" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1375,7 +1375,7 @@
       <c r="A6" s="2">
         <v>9002</v>
       </c>
-      <c r="B6" s="26">
+      <c r="B6" s="16">
         <v>46301</v>
       </c>
       <c r="C6" s="3">
@@ -1432,10 +1432,10 @@
       <c r="T6" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="U6" s="26">
+      <c r="U6" s="16">
         <v>46301</v>
       </c>
-      <c r="V6" s="25" t="s">
+      <c r="V6" s="15" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1443,7 +1443,7 @@
       <c r="A7" s="2">
         <v>9003</v>
       </c>
-      <c r="B7" s="26">
+      <c r="B7" s="16">
         <v>46301</v>
       </c>
       <c r="C7" s="3">
@@ -1500,7 +1500,7 @@
       <c r="T7" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="U7" s="26">
+      <c r="U7" s="16">
         <v>46302</v>
       </c>
       <c r="V7" s="2" t="s">
@@ -1559,80 +1559,80 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7"/>
-      <c r="Q1" s="7"/>
-      <c r="R1" s="7"/>
-      <c r="S1" s="7"/>
-      <c r="T1" s="7"/>
-      <c r="U1" s="7"/>
-      <c r="V1" s="7"/>
-      <c r="W1" s="7"/>
-      <c r="X1" s="7"/>
-      <c r="Y1" s="7"/>
-      <c r="Z1" s="7"/>
-      <c r="AA1" s="7"/>
-      <c r="AB1" s="7"/>
-      <c r="AC1" s="7"/>
-      <c r="AD1" s="7"/>
-      <c r="AE1" s="7"/>
-      <c r="AF1" s="7"/>
-      <c r="AG1" s="7"/>
-      <c r="AH1" s="7"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
+      <c r="O1" s="20"/>
+      <c r="P1" s="20"/>
+      <c r="Q1" s="20"/>
+      <c r="R1" s="20"/>
+      <c r="S1" s="20"/>
+      <c r="T1" s="20"/>
+      <c r="U1" s="20"/>
+      <c r="V1" s="20"/>
+      <c r="W1" s="20"/>
+      <c r="X1" s="20"/>
+      <c r="Y1" s="20"/>
+      <c r="Z1" s="20"/>
+      <c r="AA1" s="20"/>
+      <c r="AB1" s="20"/>
+      <c r="AC1" s="20"/>
+      <c r="AD1" s="20"/>
+      <c r="AE1" s="20"/>
+      <c r="AF1" s="20"/>
+      <c r="AG1" s="20"/>
+      <c r="AH1" s="20"/>
     </row>
     <row r="3" spans="1:34" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
-      <c r="L3" s="7"/>
-      <c r="M3" s="7"/>
-      <c r="N3" s="7"/>
-      <c r="O3" s="7"/>
-      <c r="P3" s="7"/>
-      <c r="Q3" s="7"/>
-      <c r="R3" s="7"/>
-      <c r="S3" s="7"/>
-      <c r="T3" s="7"/>
-      <c r="U3" s="7"/>
-      <c r="V3" s="7"/>
-      <c r="W3" s="7"/>
-      <c r="X3" s="7"/>
-      <c r="Y3" s="7"/>
-      <c r="Z3" s="7"/>
-      <c r="AA3" s="7"/>
-      <c r="AB3" s="7"/>
-      <c r="AC3" s="7"/>
-      <c r="AD3" s="7"/>
-      <c r="AE3" s="7"/>
-      <c r="AF3" s="7"/>
-      <c r="AG3" s="7"/>
-      <c r="AH3" s="7"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="20"/>
+      <c r="M3" s="20"/>
+      <c r="N3" s="20"/>
+      <c r="O3" s="20"/>
+      <c r="P3" s="20"/>
+      <c r="Q3" s="20"/>
+      <c r="R3" s="20"/>
+      <c r="S3" s="20"/>
+      <c r="T3" s="20"/>
+      <c r="U3" s="20"/>
+      <c r="V3" s="20"/>
+      <c r="W3" s="20"/>
+      <c r="X3" s="20"/>
+      <c r="Y3" s="20"/>
+      <c r="Z3" s="20"/>
+      <c r="AA3" s="20"/>
+      <c r="AB3" s="20"/>
+      <c r="AC3" s="20"/>
+      <c r="AD3" s="20"/>
+      <c r="AE3" s="20"/>
+      <c r="AF3" s="20"/>
+      <c r="AG3" s="20"/>
+      <c r="AH3" s="20"/>
     </row>
     <row r="4" spans="1:34" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -1757,7 +1757,7 @@
       <c r="F5" s="2">
         <v>549.9</v>
       </c>
-      <c r="G5" s="26">
+      <c r="G5" s="16">
         <v>46300</v>
       </c>
       <c r="H5" s="3">
@@ -1835,10 +1835,10 @@
       <c r="AF5" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AG5" s="26">
+      <c r="AG5" s="16">
         <v>46301</v>
       </c>
-      <c r="AH5" s="25" t="s">
+      <c r="AH5" s="15" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       <c r="F6" s="2">
         <v>499.9</v>
       </c>
-      <c r="G6" s="26">
+      <c r="G6" s="16">
         <v>46300</v>
       </c>
       <c r="H6" s="3">
@@ -1939,10 +1939,10 @@
       <c r="AF6" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AG6" s="26">
+      <c r="AG6" s="16">
         <v>46301</v>
       </c>
-      <c r="AH6" s="25" t="s">
+      <c r="AH6" s="15" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1965,7 +1965,7 @@
       <c r="F7" s="2">
         <v>499.9</v>
       </c>
-      <c r="G7" s="26">
+      <c r="G7" s="16">
         <v>46301</v>
       </c>
       <c r="H7" s="3">
@@ -1980,7 +1980,7 @@
       <c r="K7" s="4">
         <v>912345678</v>
       </c>
-      <c r="L7" s="11" t="s">
+      <c r="L7" s="7" t="s">
         <v>114</v>
       </c>
       <c r="M7" s="2" t="s">
@@ -2043,10 +2043,10 @@
       <c r="AF7" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="AG7" s="26">
+      <c r="AG7" s="16">
         <v>46301</v>
       </c>
-      <c r="AH7" s="25" t="s">
+      <c r="AH7" s="15" t="s">
         <v>42</v>
       </c>
     </row>
@@ -2069,7 +2069,7 @@
       <c r="F8" s="2">
         <v>129.9</v>
       </c>
-      <c r="G8" s="26">
+      <c r="G8" s="16">
         <v>46301</v>
       </c>
       <c r="H8" s="3">
@@ -2147,7 +2147,7 @@
       <c r="AF8" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="AG8" s="26">
+      <c r="AG8" s="16">
         <v>46302</v>
       </c>
       <c r="AH8" s="2" t="s">
@@ -2182,39 +2182,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="17" t="s">
         <v>124</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="F2" s="14"/>
+      <c r="F2" s="10"/>
     </row>
     <row r="3" spans="1:13" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
-      <c r="L3" s="7"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="20"/>
     </row>
     <row r="4" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -2247,16 +2247,16 @@
       <c r="J4" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="K4" s="15" t="s">
+      <c r="K4" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="L4" s="16"/>
+      <c r="L4" s="22"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>9001</v>
       </c>
-      <c r="B5" s="26">
+      <c r="B5" s="16">
         <v>46300</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -2280,20 +2280,20 @@
       <c r="I5" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="J5" s="20" t="s">
+      <c r="J5" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="K5" s="21" t="s">
+      <c r="K5" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="L5" s="22"/>
-      <c r="M5" s="23"/>
+      <c r="L5" s="24"/>
+      <c r="M5" s="14"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="26">
+      <c r="B6" s="16">
         <v>46301</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -2314,23 +2314,23 @@
       <c r="H6" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="I6" s="11" t="s">
+      <c r="I6" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="J6" s="20" t="s">
+      <c r="J6" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="K6" s="21" t="s">
+      <c r="K6" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="L6" s="22"/>
-      <c r="M6" s="23"/>
+      <c r="L6" s="24"/>
+      <c r="M6" s="14"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B7" s="26">
+      <c r="B7" s="16">
         <v>46301</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -2354,34 +2354,34 @@
       <c r="I7" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="J7" s="17" t="s">
+      <c r="J7" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="K7" s="19" t="s">
+      <c r="K7" s="25" t="s">
         <v>128</v>
       </c>
-      <c r="L7" s="24"/>
-      <c r="M7" s="23"/>
+      <c r="L7" s="26"/>
+      <c r="M7" s="14"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="K8" s="18"/>
-      <c r="L8" s="18"/>
+      <c r="K8" s="12"/>
+      <c r="L8" s="12"/>
     </row>
     <row r="9" spans="1:13" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="7"/>
-      <c r="K9" s="7"/>
-      <c r="L9" s="7"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="20"/>
+      <c r="K9" s="20"/>
+      <c r="L9" s="20"/>
     </row>
     <row r="10" spans="1:13" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
@@ -2484,20 +2484,20 @@
       </c>
     </row>
     <row r="16" spans="1:13" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
-      <c r="J16" s="7"/>
-      <c r="K16" s="7"/>
-      <c r="L16" s="7"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="20"/>
+      <c r="L16" s="20"/>
     </row>
     <row r="17" spans="1:12" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
@@ -2520,10 +2520,10 @@
       <c r="A18" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="26">
+      <c r="B18" s="16">
         <v>46301</v>
       </c>
-      <c r="C18" s="25" t="s">
+      <c r="C18" s="15" t="s">
         <v>57</v>
       </c>
       <c r="D18" s="3" t="s">
@@ -2537,10 +2537,10 @@
       <c r="A19" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="26">
+      <c r="B19" s="16">
         <v>46301</v>
       </c>
-      <c r="C19" s="25" t="s">
+      <c r="C19" s="15" t="s">
         <v>42</v>
       </c>
       <c r="D19" s="3" t="s">
@@ -2554,7 +2554,7 @@
       <c r="A20" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="B20" s="26">
+      <c r="B20" s="16">
         <v>46302</v>
       </c>
       <c r="C20" s="2" t="s">
@@ -2568,20 +2568,20 @@
       </c>
     </row>
     <row r="22" spans="1:12" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
+      <c r="A22" s="19" t="s">
         <v>138</v>
       </c>
-      <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="7"/>
-      <c r="I22" s="7"/>
-      <c r="J22" s="7"/>
-      <c r="K22" s="7"/>
-      <c r="L22" s="7"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="20"/>
+      <c r="H22" s="20"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="20"/>
+      <c r="L22" s="20"/>
     </row>
     <row r="23" spans="1:12" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
@@ -2704,28 +2704,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="17" t="s">
         <v>142</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
     </row>
     <row r="3" spans="1:8" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -2757,10 +2757,10 @@
       <c r="C5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="12">
+      <c r="D5" s="8">
         <v>987654321</v>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="8">
         <v>945112233</v>
       </c>
       <c r="F5" s="2" t="s">
@@ -2777,10 +2777,10 @@
       <c r="C6" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="8">
         <v>912345678</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="7" t="s">
         <v>114</v>
       </c>
       <c r="F6" s="2" t="s">
@@ -2788,16 +2788,16 @@
       </c>
     </row>
     <row r="8" spans="1:8" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
@@ -2844,16 +2844,16 @@
       </c>
     </row>
     <row r="14" spans="1:8" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="19" t="s">
         <v>149</v>
       </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="20"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
@@ -2889,16 +2889,16 @@
       </c>
     </row>
     <row r="19" spans="1:8" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="19" t="s">
         <v>151</v>
       </c>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="20"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
@@ -2945,16 +2945,16 @@
       </c>
     </row>
     <row r="25" spans="1:8" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A25" s="8" t="s">
+      <c r="A25" s="19" t="s">
         <v>153</v>
       </c>
-      <c r="B25" s="7"/>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="7"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="20"/>
     </row>
     <row r="26" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
@@ -3037,16 +3037,16 @@
       </c>
     </row>
     <row r="31" spans="1:8" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A31" s="8" t="s">
+      <c r="A31" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="B31" s="7"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7"/>
-      <c r="G31" s="7"/>
-      <c r="H31" s="7"/>
+      <c r="B31" s="20"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="20"/>
+      <c r="F31" s="20"/>
+      <c r="G31" s="20"/>
+      <c r="H31" s="20"/>
     </row>
     <row r="32" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
@@ -3072,13 +3072,13 @@
       <c r="A33" s="3">
         <v>9001</v>
       </c>
-      <c r="B33" s="26">
+      <c r="B33" s="16">
         <v>46300</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D33" s="25" t="s">
+      <c r="D33" s="15" t="s">
         <v>31</v>
       </c>
       <c r="E33" s="3">
@@ -3092,7 +3092,7 @@
       <c r="A34" s="3">
         <v>9002</v>
       </c>
-      <c r="B34" s="26">
+      <c r="B34" s="16">
         <v>46301</v>
       </c>
       <c r="C34" s="2" t="s">
@@ -3112,7 +3112,7 @@
       <c r="A35" s="3">
         <v>9003</v>
       </c>
-      <c r="B35" s="26">
+      <c r="B35" s="16">
         <v>46301</v>
       </c>
       <c r="C35" s="2" t="s">
@@ -3129,16 +3129,16 @@
       </c>
     </row>
     <row r="37" spans="1:8" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A37" s="8" t="s">
+      <c r="A37" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="B37" s="7"/>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
-      <c r="E37" s="7"/>
-      <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
-      <c r="H37" s="7"/>
+      <c r="B37" s="20"/>
+      <c r="C37" s="20"/>
+      <c r="D37" s="20"/>
+      <c r="E37" s="20"/>
+      <c r="F37" s="20"/>
+      <c r="G37" s="20"/>
+      <c r="H37" s="20"/>
     </row>
     <row r="38" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
@@ -3161,10 +3161,10 @@
       <c r="A39" s="3">
         <v>1</v>
       </c>
-      <c r="B39" s="26">
+      <c r="B39" s="16">
         <v>46301</v>
       </c>
-      <c r="C39" s="25" t="s">
+      <c r="C39" s="15" t="s">
         <v>57</v>
       </c>
       <c r="D39" s="3">
@@ -3178,10 +3178,10 @@
       <c r="A40" s="3">
         <v>2</v>
       </c>
-      <c r="B40" s="26">
+      <c r="B40" s="16">
         <v>46301</v>
       </c>
-      <c r="C40" s="25" t="s">
+      <c r="C40" s="15" t="s">
         <v>42</v>
       </c>
       <c r="D40" s="3">
@@ -3195,7 +3195,7 @@
       <c r="A41" s="3">
         <v>3</v>
       </c>
-      <c r="B41" s="26">
+      <c r="B41" s="16">
         <v>46302</v>
       </c>
       <c r="C41" s="2" t="s">
@@ -3209,16 +3209,16 @@
       </c>
     </row>
     <row r="43" spans="1:8" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A43" s="8" t="s">
+      <c r="A43" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="B43" s="7"/>
-      <c r="C43" s="7"/>
-      <c r="D43" s="7"/>
-      <c r="E43" s="7"/>
-      <c r="F43" s="7"/>
-      <c r="G43" s="7"/>
-      <c r="H43" s="7"/>
+      <c r="B43" s="20"/>
+      <c r="C43" s="20"/>
+      <c r="D43" s="20"/>
+      <c r="E43" s="20"/>
+      <c r="F43" s="20"/>
+      <c r="G43" s="20"/>
+      <c r="H43" s="20"/>
     </row>
     <row r="44" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
@@ -3247,7 +3247,7 @@
       <c r="B45" s="3">
         <v>1001</v>
       </c>
-      <c r="C45" s="13">
+      <c r="C45" s="9">
         <v>42</v>
       </c>
       <c r="D45" s="3" t="s">
@@ -3267,7 +3267,7 @@
       <c r="B46" s="3">
         <v>1002</v>
       </c>
-      <c r="C46" s="13">
+      <c r="C46" s="9">
         <v>41</v>
       </c>
       <c r="D46" s="3" t="s">
@@ -3287,7 +3287,7 @@
       <c r="B47" s="3">
         <v>1002</v>
       </c>
-      <c r="C47" s="13">
+      <c r="C47" s="9">
         <v>41</v>
       </c>
       <c r="D47" s="3" t="s">
@@ -3321,16 +3321,16 @@
       </c>
     </row>
     <row r="50" spans="1:8" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A50" s="8" t="s">
+      <c r="A50" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="B50" s="7"/>
-      <c r="C50" s="7"/>
-      <c r="D50" s="7"/>
-      <c r="E50" s="7"/>
-      <c r="F50" s="7"/>
-      <c r="G50" s="7"/>
-      <c r="H50" s="7"/>
+      <c r="B50" s="20"/>
+      <c r="C50" s="20"/>
+      <c r="D50" s="20"/>
+      <c r="E50" s="20"/>
+      <c r="F50" s="20"/>
+      <c r="G50" s="20"/>
+      <c r="H50" s="20"/>
     </row>
     <row r="51" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
@@ -3359,7 +3359,7 @@
       <c r="B52" s="3">
         <v>1001</v>
       </c>
-      <c r="C52" s="13">
+      <c r="C52" s="9">
         <v>42</v>
       </c>
       <c r="D52" s="3" t="s">
@@ -3379,7 +3379,7 @@
       <c r="B53" s="3">
         <v>1002</v>
       </c>
-      <c r="C53" s="13">
+      <c r="C53" s="9">
         <v>41</v>
       </c>
       <c r="D53" s="3" t="s">
@@ -3413,16 +3413,16 @@
       </c>
     </row>
     <row r="56" spans="1:8" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A56" s="8" t="s">
+      <c r="A56" s="19" t="s">
         <v>138</v>
       </c>
-      <c r="B56" s="7"/>
-      <c r="C56" s="7"/>
-      <c r="D56" s="7"/>
-      <c r="E56" s="7"/>
-      <c r="F56" s="7"/>
-      <c r="G56" s="7"/>
-      <c r="H56" s="7"/>
+      <c r="B56" s="20"/>
+      <c r="C56" s="20"/>
+      <c r="D56" s="20"/>
+      <c r="E56" s="20"/>
+      <c r="F56" s="20"/>
+      <c r="G56" s="20"/>
+      <c r="H56" s="20"/>
     </row>
     <row r="57" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
@@ -3448,7 +3448,7 @@
       <c r="B58" s="3">
         <v>1001</v>
       </c>
-      <c r="C58" s="13">
+      <c r="C58" s="9">
         <v>42</v>
       </c>
       <c r="D58" s="3" t="s">
@@ -3465,7 +3465,7 @@
       <c r="B59" s="3">
         <v>1002</v>
       </c>
-      <c r="C59" s="13">
+      <c r="C59" s="9">
         <v>41</v>
       </c>
       <c r="D59" s="3" t="s">
@@ -3482,7 +3482,7 @@
       <c r="B60" s="3">
         <v>1002</v>
       </c>
-      <c r="C60" s="13">
+      <c r="C60" s="9">
         <v>41</v>
       </c>
       <c r="D60" s="3" t="s">

</xml_diff>